<commit_message>
edited the docstring of MembraneSector object
</commit_message>
<xml_diff>
--- a/Data/Surface_growth_rate_data/surface_volume_data.xlsx
+++ b/Data/Surface_growth_rate_data/surface_volume_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\claud\PythonProject\iamb-student-folders\iamb-folder-template\40-49_Experiments\40_Raw_Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\claud\PythonProject\mcPAModelpy\PAModelpy\Data\Surface_growth_rate_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A04F8F66-D034-4A22-B70E-4E1BC9DA3744}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF812D05-5539-4E84-A986-06DD59C0462F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Szenk_Paper" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="bacteria shape" sheetId="6" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="1" hidden="1">Heinemann_paper!$L$1:$L$25</definedName>
+    <definedName name="ExternalData_1" localSheetId="1" hidden="1">Heinemann_paper!$N$1:$N$25</definedName>
     <definedName name="ExterneDaten_2" localSheetId="1" hidden="1">Heinemann_paper!$A$1:$D$25</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -133,7 +133,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="42">
   <si>
     <t>Growth Rate</t>
   </si>
@@ -246,13 +246,19 @@
     <t>Cell width-2x [um]</t>
   </si>
   <si>
-    <t>S/V [1/m]</t>
-  </si>
-  <si>
     <t>Cell volume [fl]</t>
   </si>
   <si>
     <t>single_cell_volume[fl]</t>
+  </si>
+  <si>
+    <t>Cell volume [L]</t>
+  </si>
+  <si>
+    <t>Inner membrane surface [m2]</t>
+  </si>
+  <si>
+    <t>S/V [um2/fL]</t>
   </si>
 </sst>
 </file>
@@ -356,7 +362,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -374,11 +380,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="13">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
@@ -2736,7 +2749,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Heinemann_paper!$K$2:$K$25</c:f>
+              <c:f>Heinemann_paper!$L$2:$L$25</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="24"/>
@@ -3236,7 +3249,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Heinemann_paper!$M$2:$M$23</c:f>
+              <c:f>Heinemann_paper!$O$2:$O$23</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="22"/>
@@ -3771,7 +3784,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Heinemann_paper!$L$2:$L$25</c:f>
+              <c:f>Heinemann_paper!$N$2:$N$25</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="24"/>
@@ -7539,7 +7552,7 @@
       <xdr:rowOff>79561</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>498662</xdr:colOff>
       <xdr:row>42</xdr:row>
       <xdr:rowOff>155761</xdr:rowOff>
@@ -7575,7 +7588,7 @@
       <xdr:rowOff>180414</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>963706</xdr:colOff>
       <xdr:row>58</xdr:row>
       <xdr:rowOff>66114</xdr:rowOff>
@@ -8394,8 +8407,8 @@
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="ExterneDaten_2" connectionId="2" xr16:uid="{C1D4B7B6-36CA-4149-97AA-8051E4442D38}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
-  <queryTableRefresh nextId="18" unboundColumnsRight="7">
-    <queryTableFields count="11">
+  <queryTableRefresh nextId="20" unboundColumnsRight="9">
+    <queryTableFields count="13">
       <queryTableField id="1" name="Growth condition" tableColumnId="1"/>
       <queryTableField id="2" name="Growth Rate  [1/h].1" tableColumnId="2"/>
       <queryTableField id="3" name="Cell Length [um] " tableColumnId="3"/>
@@ -8406,7 +8419,9 @@
       <queryTableField id="12" dataBound="0" tableColumnId="12"/>
       <queryTableField id="11" dataBound="0" tableColumnId="11"/>
       <queryTableField id="8" dataBound="0" tableColumnId="8"/>
+      <queryTableField id="19" dataBound="0" tableColumnId="10"/>
       <queryTableField id="15" dataBound="0" tableColumnId="15"/>
+      <queryTableField id="18" dataBound="0" tableColumnId="9"/>
     </queryTableFields>
   </queryTableRefresh>
 </queryTable>
@@ -8434,33 +8449,39 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{31A44E15-1885-4BAD-9771-9733731DD5A2}" name="Heinemann_cell_length_width_data__2" displayName="Heinemann_cell_length_width_data__2" ref="A1:K25" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:K25" xr:uid="{31A44E15-1885-4BAD-9771-9733731DD5A2}"/>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{8DEE30FE-C545-4C1E-B5FE-C86621848749}" uniqueName="1" name="Growth condition" queryTableFieldId="1" dataDxfId="10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{31A44E15-1885-4BAD-9771-9733731DD5A2}" name="Heinemann_cell_length_width_data__2" displayName="Heinemann_cell_length_width_data__2" ref="A1:M25" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:M25" xr:uid="{31A44E15-1885-4BAD-9771-9733731DD5A2}"/>
+  <tableColumns count="13">
+    <tableColumn id="1" xr3:uid="{8DEE30FE-C545-4C1E-B5FE-C86621848749}" uniqueName="1" name="Growth condition" queryTableFieldId="1" dataDxfId="12"/>
     <tableColumn id="2" xr3:uid="{13BEBAE8-C8A7-4E54-87F7-2BADEC8C25D4}" uniqueName="2" name="Growth Rate  [1/h].1" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{67234470-2606-4547-AF13-B61BB0C4735E}" uniqueName="3" name="Cell Length [um] " queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{2A2E582D-13A5-4D73-9B44-B2F97C7E7B57}" uniqueName="4" name="Cell Width [um]" queryTableFieldId="4"/>
     <tableColumn id="5" xr3:uid="{6C636F70-6094-4608-ADB9-397A88C87196}" uniqueName="5" name="a [um]" queryTableFieldId="5">
       <calculatedColumnFormula>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{B29E6144-153B-43C8-8B1C-A95BE6E17B48}" uniqueName="6" name="b [um]" queryTableFieldId="6" dataDxfId="9">
+    <tableColumn id="6" xr3:uid="{B29E6144-153B-43C8-8B1C-A95BE6E17B48}" uniqueName="6" name="b [um]" queryTableFieldId="6" dataDxfId="11">
       <calculatedColumnFormula>Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{49ABCC3A-8D16-41FC-898A-82F743E84101}" uniqueName="7" name="Cell Surface [um2]" queryTableFieldId="7" dataDxfId="8">
+    <tableColumn id="7" xr3:uid="{49ABCC3A-8D16-41FC-898A-82F743E84101}" uniqueName="7" name="Cell Surface [um2]" queryTableFieldId="7" dataDxfId="10">
       <calculatedColumnFormula>2*PI()*(Heinemann_cell_length_width_data__2[[#This Row],[a '[um']]]/2)*Heinemann_cell_length_width_data__2[[#This Row],[b '[um']]]+4*PI()*(Heinemann_cell_length_width_data__2[[#This Row],[a '[um']]]/2)^2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{193ECAAE-58D2-41E3-92F8-BC91BCFC1547}" uniqueName="12" name="Cell  length-2x [um]" queryTableFieldId="12" dataDxfId="7">
+    <tableColumn id="12" xr3:uid="{193ECAAE-58D2-41E3-92F8-BC91BCFC1547}" uniqueName="12" name="Cell  length-2x [um]" queryTableFieldId="12" dataDxfId="9">
       <calculatedColumnFormula>Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-0.4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{3B53D017-4125-4E0C-A121-61AFACAF77D2}" uniqueName="11" name="Cell width-2x [um]" queryTableFieldId="11" dataDxfId="6">
+    <tableColumn id="11" xr3:uid="{3B53D017-4125-4E0C-A121-61AFACAF77D2}" uniqueName="11" name="Cell width-2x [um]" queryTableFieldId="11" dataDxfId="8">
       <calculatedColumnFormula>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]-0.4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{BCB42941-9B05-4976-A177-3DEC2CD5BC2A}" uniqueName="8" name="Inner membrane surface [um2]" queryTableFieldId="8" dataDxfId="5">
+    <tableColumn id="8" xr3:uid="{BCB42941-9B05-4976-A177-3DEC2CD5BC2A}" uniqueName="8" name="Inner membrane surface [um2]" queryTableFieldId="8" dataDxfId="7">
       <calculatedColumnFormula>2*PI()*(Heinemann_cell_length_width_data__2[[#This Row],[Cell width-2x '[um']]]/2)*Heinemann_cell_length_width_data__2[[#This Row],[Cell  length-2x '[um']]]+4*PI()*(Heinemann_cell_length_width_data__2[[#This Row],[Cell width-2x '[um']]]/2)^2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{1EF9F28C-5548-4C71-9347-CA143F899338}" uniqueName="15" name="Cell volume [fl]" queryTableFieldId="15" dataDxfId="4">
+    <tableColumn id="10" xr3:uid="{61022530-D945-4339-9351-372633BFD53A}" uniqueName="10" name="Inner membrane surface [m2]" queryTableFieldId="19" dataDxfId="0">
+      <calculatedColumnFormula>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="15" xr3:uid="{1EF9F28C-5548-4C71-9347-CA143F899338}" uniqueName="15" name="Cell volume [fl]" queryTableFieldId="15" dataDxfId="6">
       <calculatedColumnFormula>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="9" xr3:uid="{78351E1D-2325-4CB4-A8C8-E40E31CE1B71}" uniqueName="9" name="Cell volume [L]" queryTableFieldId="18" dataDxfId="1">
+      <calculatedColumnFormula>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -8468,11 +8489,11 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{71844E39-6B65-4C9F-9F87-9DD0BA592C0C}" name="Heinemann_cell_length_width_data__34" displayName="Heinemann_cell_length_width_data__34" ref="L1:M25" tableType="queryTable" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2">
-  <autoFilter ref="L1:M25" xr:uid="{71844E39-6B65-4C9F-9F87-9DD0BA592C0C}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{71844E39-6B65-4C9F-9F87-9DD0BA592C0C}" name="Heinemann_cell_length_width_data__34" displayName="Heinemann_cell_length_width_data__34" ref="N1:O25" tableType="queryTable" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+  <autoFilter ref="N1:O25" xr:uid="{71844E39-6B65-4C9F-9F87-9DD0BA592C0C}"/>
   <tableColumns count="2">
-    <tableColumn id="5" xr3:uid="{18E7EA0B-5A3F-4283-9D61-3FE21071CAA5}" uniqueName="5" name="single_cell_volume[fl]" queryTableFieldId="5" dataDxfId="1"/>
-    <tableColumn id="10" xr3:uid="{E1B4AFAC-E374-4EA0-91DD-5A8BB80369E4}" uniqueName="10" name="S/V [1/m]" queryTableFieldId="10" dataDxfId="0">
+    <tableColumn id="5" xr3:uid="{18E7EA0B-5A3F-4283-9D61-3FE21071CAA5}" uniqueName="5" name="single_cell_volume[fl]" queryTableFieldId="5" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{E1B4AFAC-E374-4EA0-91DD-5A8BB80369E4}" uniqueName="10" name="S/V [um2/fL]" queryTableFieldId="10" dataDxfId="2">
       <calculatedColumnFormula>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -8818,7 +8839,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB5093F8-ACFF-4697-A1E7-BF5FEA75B594}">
-  <dimension ref="A1:M87"/>
+  <dimension ref="A1:O87"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
@@ -8829,11 +8850,12 @@
     <col min="7" max="7" width="16.140625" customWidth="1"/>
     <col min="8" max="8" width="21" customWidth="1"/>
     <col min="9" max="9" width="16.140625" customWidth="1"/>
-    <col min="10" max="10" width="22.85546875" customWidth="1"/>
-    <col min="12" max="12" width="21.140625" style="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="33.28515625" customWidth="1"/>
+    <col min="12" max="13" width="27.28515625" customWidth="1"/>
+    <col min="14" max="14" width="21.140625" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>28</v>
       </c>
@@ -8865,16 +8887,22 @@
         <v>33</v>
       </c>
       <c r="K1" t="s">
+        <v>40</v>
+      </c>
+      <c r="L1" t="s">
+        <v>37</v>
+      </c>
+      <c r="M1" t="s">
+        <v>39</v>
+      </c>
+      <c r="N1" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="L1" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="M1" s="10" t="s">
-        <v>37</v>
+      <c r="O1" s="10" t="s">
+        <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -8912,18 +8940,26 @@
         <v>12.44070690821558</v>
       </c>
       <c r="K2">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>1.2440706908215579E-11</v>
+      </c>
+      <c r="L2">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>4.6013860399578501</v>
       </c>
-      <c r="L2" s="10">
+      <c r="M2" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>4.6013860399578507E-15</v>
+      </c>
+      <c r="N2" s="10">
         <v>4.4000000000000004</v>
       </c>
-      <c r="M2" s="10">
+      <c r="O2" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>2.7036868456986798</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -8961,18 +8997,26 @@
         <v>12.88052987971815</v>
       </c>
       <c r="K3">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>1.2880529879718149E-11</v>
+      </c>
+      <c r="L3">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>4.6694538807856283</v>
       </c>
-      <c r="L3" s="10">
+      <c r="M3" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>4.6694538807856284E-15</v>
+      </c>
+      <c r="N3" s="10">
         <v>3.9</v>
       </c>
-      <c r="M3" s="10">
+      <c r="O3" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>2.7584660237721463</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -9010,18 +9054,26 @@
         <v>14.514158059584847</v>
       </c>
       <c r="K4">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>1.4514158059584847E-11</v>
+      </c>
+      <c r="L4">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>5.3014376029327757</v>
       </c>
-      <c r="L4" s="10">
+      <c r="M4" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>5.3014376029327759E-15</v>
+      </c>
+      <c r="N4" s="10">
         <v>4</v>
       </c>
-      <c r="M4" s="10">
+      <c r="O4" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>2.7377777777777785</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -9059,18 +9111,26 @@
         <v>15.205308443374602</v>
       </c>
       <c r="K5">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>1.5205308443374603E-11</v>
+      </c>
+      <c r="L5">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>5.6548667764616276</v>
       </c>
-      <c r="L5" s="10">
+      <c r="M5" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>5.6548667764616284E-15</v>
+      </c>
+      <c r="N5" s="10">
         <v>4.0999999999999996</v>
       </c>
-      <c r="M5" s="10">
+      <c r="O5" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>2.6888888888888896</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -9108,18 +9168,26 @@
         <v>14.514158059584847</v>
       </c>
       <c r="K6">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>1.4514158059584847E-11</v>
+      </c>
+      <c r="L6">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>5.3014376029327757</v>
       </c>
-      <c r="L6" s="10">
+      <c r="M6" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>5.3014376029327759E-15</v>
+      </c>
+      <c r="N6" s="10">
         <v>3.9</v>
       </c>
-      <c r="M6" s="10">
+      <c r="O6" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>2.7377777777777785</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -9157,18 +9225,26 @@
         <v>6.7858401317539521</v>
       </c>
       <c r="K7">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>6.7858401317539517E-12</v>
+      </c>
+      <c r="L7">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>2.1488493750554185</v>
       </c>
-      <c r="L7" s="10">
+      <c r="M7" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>2.1488493750554186E-15</v>
+      </c>
+      <c r="N7" s="10">
         <v>2.4</v>
       </c>
-      <c r="M7" s="10">
+      <c r="O7" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>3.1578947368421049</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -9206,18 +9282,26 @@
         <v>5.9376101152847092</v>
       </c>
       <c r="K8">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>5.937610115284709E-12</v>
+      </c>
+      <c r="L8">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>1.9323412813455221</v>
       </c>
-      <c r="L8" s="10">
+      <c r="M8" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>1.9323412813455221E-15</v>
+      </c>
+      <c r="N8" s="10">
         <v>2.4</v>
       </c>
-      <c r="M8" s="10">
+      <c r="O8" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>3.0727543693266495</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -9255,18 +9339,26 @@
         <v>5.0579641722795676</v>
       </c>
       <c r="K9">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>5.0579641722795677E-12</v>
+      </c>
+      <c r="L9">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>1.5522085702611572</v>
       </c>
-      <c r="L9" s="10">
+      <c r="M9" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>1.5522085702611574E-15</v>
+      </c>
+      <c r="N9" s="10">
         <v>1.9</v>
       </c>
-      <c r="M9" s="10">
+      <c r="O9" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>3.2585596221959858</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -9304,18 +9396,26 @@
         <v>11.309733552923255</v>
       </c>
       <c r="K10">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>1.1309733552923255E-11</v>
+      </c>
+      <c r="L10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>3.8997636806561289</v>
       </c>
-      <c r="L10" s="10">
+      <c r="M10" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>3.899763680656129E-15</v>
+      </c>
+      <c r="N10" s="10">
         <v>3.2</v>
       </c>
-      <c r="M10" s="10">
+      <c r="O10" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>2.9001074113856076</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -9353,18 +9453,26 @@
         <v>10.681415022205293</v>
       </c>
       <c r="K11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>1.0681415022205293E-11</v>
+      </c>
+      <c r="L11">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>3.5918876006043297</v>
       </c>
-      <c r="L11" s="10">
+      <c r="M11" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>3.5918876006043303E-15</v>
+      </c>
+      <c r="N11" s="10">
         <v>3</v>
       </c>
-      <c r="M11" s="10">
+      <c r="O11" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>2.973760932944606</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -9402,18 +9510,26 @@
         <v>9.0477868423386045</v>
       </c>
       <c r="K12">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>9.0477868423386039E-12</v>
+      </c>
+      <c r="L12">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>3.0085985645878255</v>
       </c>
-      <c r="L12" s="10">
+      <c r="M12" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>3.0085985645878256E-15</v>
+      </c>
+      <c r="N12" s="10">
         <v>2.9</v>
       </c>
-      <c r="M12" s="10">
+      <c r="O12" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>3.0073094326487988</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -9451,18 +9567,26 @@
         <v>6.7858401317539521</v>
       </c>
       <c r="K13">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>6.7858401317539517E-12</v>
+      </c>
+      <c r="L13">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>2.1488493750554185</v>
       </c>
-      <c r="L13" s="10">
+      <c r="M13" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>2.1488493750554186E-15</v>
+      </c>
+      <c r="N13" s="10">
         <v>2.2999999999999998</v>
       </c>
-      <c r="M13" s="10">
+      <c r="O13" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>3.1578947368421049</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -9500,18 +9624,26 @@
         <v>4.5238934211693023</v>
       </c>
       <c r="K14">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>4.5238934211693019E-12</v>
+      </c>
+      <c r="L14">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>1.4660765716752369</v>
       </c>
-      <c r="L14" s="10">
+      <c r="M14" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>1.466076571675237E-15</v>
+      </c>
+      <c r="N14" s="10">
         <v>2.1</v>
       </c>
-      <c r="M14" s="10">
+      <c r="O14" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>3.0857142857142859</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -9549,18 +9681,26 @@
         <v>5.9376101152847092</v>
       </c>
       <c r="K15">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>5.937610115284709E-12</v>
+      </c>
+      <c r="L15">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>1.9323412813455221</v>
       </c>
-      <c r="L15" s="10">
+      <c r="M15" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>1.9323412813455221E-15</v>
+      </c>
+      <c r="N15" s="10">
         <v>2.4</v>
       </c>
-      <c r="M15" s="10">
+      <c r="O15" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>3.0727543693266495</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -9598,18 +9738,26 @@
         <v>9.3305301811616861</v>
       </c>
       <c r="K16">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>9.3305301811616861E-12</v>
+      </c>
+      <c r="L16">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>3.141330854201994</v>
       </c>
-      <c r="L16" s="10">
+      <c r="M16" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>3.1413308542019942E-15</v>
+      </c>
+      <c r="N16" s="10">
         <v>2.9</v>
       </c>
-      <c r="M16" s="10">
+      <c r="O16" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>2.9702475206267192</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -9647,18 +9795,26 @@
         <v>8.765043503515523</v>
       </c>
       <c r="K17">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>8.7650435035155232E-12</v>
+      </c>
+      <c r="L17">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>2.8758662749736565</v>
       </c>
-      <c r="L17" s="10">
+      <c r="M17" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>2.8758662749736566E-15</v>
+      </c>
+      <c r="N17" s="10">
         <v>2.8</v>
       </c>
-      <c r="M17" s="10">
+      <c r="O17" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>3.0477924442421482</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -9696,18 +9852,26 @@
         <v>9.6132735199847676</v>
       </c>
       <c r="K18">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>9.6132735199847667E-12</v>
+      </c>
+      <c r="L18">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>3.2740631438161625</v>
       </c>
-      <c r="L18" s="10">
+      <c r="M18" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>3.2740631438161628E-15</v>
+      </c>
+      <c r="N18" s="10">
         <v>3.1</v>
       </c>
-      <c r="M18" s="10">
+      <c r="O18" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>2.9361906284983212</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>19</v>
       </c>
@@ -9745,18 +9909,26 @@
         <v>9.0477868423386045</v>
       </c>
       <c r="K19">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>9.0477868423386039E-12</v>
+      </c>
+      <c r="L19">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>3.0085985645878255</v>
       </c>
-      <c r="L19" s="10">
+      <c r="M19" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>3.0085985645878256E-15</v>
+      </c>
+      <c r="N19" s="10">
         <v>2.8</v>
       </c>
-      <c r="M19" s="10">
+      <c r="O19" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>3.0073094326487988</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>22</v>
       </c>
@@ -9794,18 +9966,26 @@
         <v>7.2884949563283197</v>
       </c>
       <c r="K20">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>7.2884949563283196E-12</v>
+      </c>
+      <c r="L20">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>2.3750440461138838</v>
       </c>
-      <c r="L20" s="10">
+      <c r="M20" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>2.3750440461138839E-15</v>
+      </c>
+      <c r="N20" s="10">
         <v>2.6</v>
       </c>
-      <c r="M20" s="10">
+      <c r="O20" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>3.0687830687830684</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>23</v>
       </c>
@@ -9843,18 +10023,26 @@
         <v>4.9008845396000771</v>
       </c>
       <c r="K21">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>4.9008845396000769E-12</v>
+      </c>
+      <c r="L21">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>1.6231562043547263</v>
       </c>
-      <c r="L21" s="10">
+      <c r="M21" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>1.6231562043547264E-15</v>
+      </c>
+      <c r="N21" s="10">
         <v>2.4</v>
       </c>
-      <c r="M21" s="10">
+      <c r="O21" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>3.0193548387096776</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>24</v>
       </c>
@@ -9892,18 +10080,26 @@
         <v>4.5238934211693023</v>
       </c>
       <c r="K22">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>4.5238934211693019E-12</v>
+      </c>
+      <c r="L22">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>1.4660765716752369</v>
       </c>
-      <c r="L22" s="10">
+      <c r="M22" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>1.466076571675237E-15</v>
+      </c>
+      <c r="N22" s="10">
         <v>2.2000000000000002</v>
       </c>
-      <c r="M22" s="10">
+      <c r="O22" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>3.0857142857142859</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>25</v>
       </c>
@@ -9941,18 +10137,26 @@
         <v>5.2778756580308528</v>
       </c>
       <c r="K23">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>5.2778756580308527E-12</v>
+      </c>
+      <c r="L23">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>1.6472417480322485</v>
       </c>
-      <c r="L23" s="10">
+      <c r="M23" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>1.6472417480322486E-15</v>
+      </c>
+      <c r="N23" s="10">
         <v>2.1</v>
       </c>
-      <c r="M23" s="10">
+      <c r="O23" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>3.2040686586141125</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>20</v>
       </c>
@@ -9990,18 +10194,26 @@
         <v>4.1783182292744252</v>
       </c>
       <c r="K24">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>4.1783182292744248E-12</v>
+      </c>
+      <c r="L24">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>1.1720758591767924</v>
       </c>
-      <c r="L24" s="10">
+      <c r="M24" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>1.1720758591767923E-15</v>
+      </c>
+      <c r="N24" s="10">
         <v>1.5</v>
       </c>
-      <c r="M24" s="10">
+      <c r="O24" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>3.5648872012508366</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>21</v>
       </c>
@@ -10039,13 +10251,21 @@
         <v>7.2256631032565224</v>
       </c>
       <c r="K25">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</f>
+        <v>7.2256631032565223E-12</v>
+      </c>
+      <c r="L25">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</f>
         <v>1.8985691603194312</v>
       </c>
-      <c r="L25" s="10">
+      <c r="M25" s="11">
+        <f>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</f>
+        <v>1.8985691603194312E-15</v>
+      </c>
+      <c r="N25" s="10">
         <v>1.6</v>
       </c>
-      <c r="M25" s="10">
+      <c r="O25" s="10">
         <f>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</f>
         <v>3.80584666298952</v>
       </c>

</xml_diff>

<commit_message>
changed the parametrization of fraction f. Instead of calculating using pure membrane area, surface to volume ratio was used
</commit_message>
<xml_diff>
--- a/Data/Surface_growth_rate_data/surface_volume_data.xlsx
+++ b/Data/Surface_growth_rate_data/surface_volume_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\claud\PythonProject\mcPAModelpy\PAModelpy\Data\Surface_growth_rate_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF812D05-5539-4E84-A986-06DD59C0462F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3841D00-4712-460C-BF4E-3240CEBCF1EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -387,10 +387,7 @@
   </cellStyles>
   <dxfs count="13">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -402,7 +399,10 @@
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -8474,13 +8474,13 @@
     <tableColumn id="8" xr3:uid="{BCB42941-9B05-4976-A177-3DEC2CD5BC2A}" uniqueName="8" name="Inner membrane surface [um2]" queryTableFieldId="8" dataDxfId="7">
       <calculatedColumnFormula>2*PI()*(Heinemann_cell_length_width_data__2[[#This Row],[Cell width-2x '[um']]]/2)*Heinemann_cell_length_width_data__2[[#This Row],[Cell  length-2x '[um']]]+4*PI()*(Heinemann_cell_length_width_data__2[[#This Row],[Cell width-2x '[um']]]/2)^2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{61022530-D945-4339-9351-372633BFD53A}" uniqueName="10" name="Inner membrane surface [m2]" queryTableFieldId="19" dataDxfId="0">
+    <tableColumn id="10" xr3:uid="{61022530-D945-4339-9351-372633BFD53A}" uniqueName="10" name="Inner membrane surface [m2]" queryTableFieldId="19" dataDxfId="6">
       <calculatedColumnFormula>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]*0.000000000001</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{1EF9F28C-5548-4C71-9347-CA143F899338}" uniqueName="15" name="Cell volume [fl]" queryTableFieldId="15" dataDxfId="6">
+    <tableColumn id="15" xr3:uid="{1EF9F28C-5548-4C71-9347-CA143F899338}" uniqueName="15" name="Cell volume [fl]" queryTableFieldId="15" dataDxfId="5">
       <calculatedColumnFormula>Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^2*PI()/4*(Heinemann_cell_length_width_data__2[[#This Row],[Cell Length '[um'] ]]-Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]])+(PI()*Heinemann_cell_length_width_data__2[[#This Row],[Cell Width '[um']]]^3/6)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{78351E1D-2325-4CB4-A8C8-E40E31CE1B71}" uniqueName="9" name="Cell volume [L]" queryTableFieldId="18" dataDxfId="1">
+    <tableColumn id="9" xr3:uid="{78351E1D-2325-4CB4-A8C8-E40E31CE1B71}" uniqueName="9" name="Cell volume [L]" queryTableFieldId="18" dataDxfId="4">
       <calculatedColumnFormula>Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]*0.000000000000001</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -8489,11 +8489,11 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{71844E39-6B65-4C9F-9F87-9DD0BA592C0C}" name="Heinemann_cell_length_width_data__34" displayName="Heinemann_cell_length_width_data__34" ref="N1:O25" tableType="queryTable" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{71844E39-6B65-4C9F-9F87-9DD0BA592C0C}" name="Heinemann_cell_length_width_data__34" displayName="Heinemann_cell_length_width_data__34" ref="N1:O25" tableType="queryTable" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2">
   <autoFilter ref="N1:O25" xr:uid="{71844E39-6B65-4C9F-9F87-9DD0BA592C0C}"/>
   <tableColumns count="2">
-    <tableColumn id="5" xr3:uid="{18E7EA0B-5A3F-4283-9D61-3FE21071CAA5}" uniqueName="5" name="single_cell_volume[fl]" queryTableFieldId="5" dataDxfId="3"/>
-    <tableColumn id="10" xr3:uid="{E1B4AFAC-E374-4EA0-91DD-5A8BB80369E4}" uniqueName="10" name="S/V [um2/fL]" queryTableFieldId="10" dataDxfId="2">
+    <tableColumn id="5" xr3:uid="{18E7EA0B-5A3F-4283-9D61-3FE21071CAA5}" uniqueName="5" name="single_cell_volume[fl]" queryTableFieldId="5" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{E1B4AFAC-E374-4EA0-91DD-5A8BB80369E4}" uniqueName="10" name="S/V [um2/fL]" queryTableFieldId="10" dataDxfId="0">
       <calculatedColumnFormula>Heinemann_cell_length_width_data__2[[#This Row],[Inner membrane surface '[um2']]]/Heinemann_cell_length_width_data__2[[#This Row],[Cell volume '[fl']]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>

</xml_diff>